<commit_message>
Record team-verified IndiaMart listings for ICU Medical pumps (slide 2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014jxHyvpwsKVbJ3RxrkkV1k
</commit_message>
<xml_diff>
--- a/Infusion_Pumps_India/Infusion_Pump_Classification_India_Slide2.xlsx
+++ b/Infusion_Pumps_India/Infusion_Pump_Classification_India_Slide2.xlsx
@@ -2090,12 +2090,12 @@
       </c>
       <c r="L16" s="13" t="inlineStr">
         <is>
-          <t>IndiaMart is blocked for automated access - project team to confirm the listing opens.</t>
+          <t>IndiaMart listing verified by project team (Oct-2026): seller Nature's Global Service, New Delhi, Rs 30,000; image shows a Graseby 2000.</t>
         </is>
       </c>
       <c r="M16" s="13" t="inlineStr">
         <is>
-          <t>Honmed_Graseby_2100.jpg (IndiaMart: team check)</t>
+          <t>IndiaMart_Graseby_2000_team_check.jpg; Honmed_Graseby_2100.jpg</t>
         </is>
       </c>
     </row>
@@ -2155,10 +2155,14 @@
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="L17" s="13" t="inlineStr"/>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>IndiaMart listing verified by project team: seller Apex Medical India (Mark.Inc), Lucknow, Rs 30,000; pump screen shows WEIGHT / DRUG MASS fields (body-weight mode).</t>
+        </is>
+      </c>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>Honmed_Graseby_2100.jpg</t>
+          <t>Honmed_Graseby_2100.jpg; IndiaMart_Graseby_2100_team_check.jpg</t>
         </is>
       </c>
     </row>
@@ -2220,12 +2224,12 @@
       </c>
       <c r="L18" s="13" t="inlineStr">
         <is>
-          <t>Only India evidence is the IndiaMart listing (blocked here) - team to confirm. ICU Medical has no India product website.</t>
+          <t>IndiaMart listing verified by project team: seller Apex Medical India (Mark.Inc), Lucknow, Rs 1,80,000; product photo shows the 'PharmGuard Medication Safety' start screen (drug library). ICU Medical has no India product website.</t>
         </is>
       </c>
       <c r="M18" s="13" t="inlineStr">
         <is>
-          <t>ICU_Global_Medfusion_4000.jpg (IndiaMart: team check)</t>
+          <t>IndiaMart_Medfusion_4000_team_check.jpg; ICU_Global_Medfusion_4000.jpg</t>
         </is>
       </c>
     </row>
@@ -2287,12 +2291,12 @@
       </c>
       <c r="L19" s="13" t="inlineStr">
         <is>
-          <t>Some non-Indian distributors list a newer 'Graseby 1200' with a 2,000-drug library - not seen on Indian sites.</t>
+          <t>Medikabazaar (Rs 48,825) is primary - its photo shows the Graseby 1200 volumetric pump. IndiaMart listing (team-verified: Horizon Medical Technologies, New Delhi, Rs 55,000) is titled Graseby 1200 but its photo shows a Graseby 2000 SYRINGE pump - use as supporting only. Some non-Indian distributors list a newer 'Graseby 1200' with a 2,000-drug library - not seen on Indian sites.</t>
         </is>
       </c>
       <c r="M19" s="13" t="inlineStr">
         <is>
-          <t>Medikabazaar_Graseby_1200.jpg; Graseby_1200_India_brochure_Hospimax_p2.jpg; ..._p3.jpg</t>
+          <t>Medikabazaar_Graseby_1200.jpg; IndiaMart_Graseby_1200_team_check.jpg; Graseby_1200_India_brochure_Hospimax_p2.jpg; ..._p3.jpg</t>
         </is>
       </c>
     </row>
@@ -3372,12 +3376,12 @@
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>KEEP (peach) - team to verify</t>
+          <t>KEEP (peach) - team-verified</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>IndiaMart blocked for automated access here</t>
+          <t>Apex Medical India, Lucknow, Rs 1,80,000</t>
         </is>
       </c>
     </row>
@@ -3436,12 +3440,12 @@
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>ADDED (peach) - team to verify</t>
+          <t>ADDED (peach) - team-verified</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>Sample had no URL for Graseby 2000/2100</t>
+          <t>Nature's Global Service, New Delhi, Rs 30,000. Sample had no URL for Graseby 2000/2100</t>
         </is>
       </c>
     </row>
@@ -3500,10 +3504,14 @@
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>ADDED (peach) - team to verify</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr"/>
+          <t>ADDED (peach) - team-verified</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Apex Medical India, Lucknow, Rs 30,000</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
@@ -3528,12 +3536,12 @@
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>KEEP (peach) - team to verify</t>
+          <t>SUPPORTING ONLY (peach) - team-verified</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Tracking parameter removed</t>
+          <t>Horizon Medical Technologies, New Delhi, Rs 55,000. CAUTION: listing photo shows a Graseby 2000 syringe pump - show Medikabazaar to clients instead</t>
         </is>
       </c>
     </row>
@@ -3560,12 +3568,12 @@
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>KEEP (peach)</t>
+          <t>KEEP (peach) - PRIMARY</t>
         </is>
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
-          <t>Tracking parameters removed; page shows price, no drug library</t>
+          <t>Tracking parameters removed; photo shows the 1200 volumetric pump; Rs 48,825</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3771,7 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>7. LIMITATION: IndiaMart blocks automated access from this environment (HTTP 429), and smiths-medical.com (incl. its /en-in pages) was unreachable. IndiaMart links need a manual check by the project team.</t>
+          <t>7. IndiaMart blocks automated access from this environment (HTTP 429); all four IndiaMart listings (Medfusion 4000, Graseby 2000, 2100, 1200) were verified manually by the project team (screenshots in evidence/). smiths-medical.com (incl. /en-in) was unreachable.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Slide 2: keep Graseby under ICU Medical and include Terumo 730 models per team decision
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014jxHyvpwsKVbJ3RxrkkV1k
</commit_message>
<xml_diff>
--- a/Infusion_Pumps_India/Infusion_Pump_Classification_India_Slide2.xlsx
+++ b/Infusion_Pumps_India/Infusion_Pump_Classification_India_Slide2.xlsx
@@ -836,8 +836,7 @@
       <c r="J6" s="13" t="inlineStr">
         <is>
           <t>- TE-SS730 &amp; TE-LM730: Smart -&gt; Standard (brochure: 'Standard pumps without IT functions'; library mode is 830-only)
-- TE-SS830 &amp; TE-LM830 Connected confirmed (built-in wireless LAN)
-- 730 models appear only in the India-hosted brochure: confirm they are still sold</t>
+- TE-SS830 &amp; TE-LM830 Connected confirmed (built-in wireless LAN)</t>
         </is>
       </c>
     </row>
@@ -964,8 +963,7 @@
       <c r="I9" s="15" t="n"/>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>- No change in classification (Graseby 2000/2100 &amp; 1200 Standard; Medfusion 4000 Connected; all distributor-only, peach)
-- Flag: ICU's FY2025 10-K does not mention Graseby, and graseby.com is now run by Lianying Graseby Medical (China): confirm who supplies Graseby in India</t>
+          <t>- No change in classification (Graseby 2000/2100 &amp; 1200 Standard; Medfusion 4000 Connected; all distributor-only, peach)</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1174,7 @@
       </c>
       <c r="L2" s="13" t="inlineStr">
         <is>
-          <t>Shown only in the brochure hosted on terumoindia.com (brochure dated Aug-2018). The India web page text names only the Smart pumps - confirm TE-SS730 is still actively sold in India.</t>
+          <t>Shown in the brochure hosted on terumoindia.com (Aug-2018 edition); the India web page text names only the Smart pumps. Included on the slide per project team decision.</t>
         </is>
       </c>
       <c r="M2" s="13" t="inlineStr">
@@ -1310,7 +1308,7 @@
       </c>
       <c r="L4" s="13" t="inlineStr">
         <is>
-          <t>Same caveat as TE-SS730: confirm it is still actively sold in India.</t>
+          <t>Same as TE-SS730: India-hosted brochure; included per project team decision.</t>
         </is>
       </c>
       <c r="M4" s="13" t="inlineStr">
@@ -3757,14 +3755,14 @@
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>5. Terumo TE-SS730 / TE-LM730 appear only in the India-hosted brochure (2018 edition); the India web page text mentions only the Smart (830) pumps.</t>
+          <t>5. Terumo TE-SS730 / TE-LM730 appear in the India-hosted brochure (2018 edition) but not in the India web page text; included per project team decision.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>6. Graseby ownership flag: ICU Medical's FY2025 10-K describes Medfusion 4000 but does not mention Graseby, and graseby.com is now operated by Lianying Graseby Medical (Zhejiang, China). Indian listings still say 'Smiths Medical Graseby'. Confirm Graseby's current owner / India supplier before keeping it under ICU Medical.</t>
+          <t>6. Graseby: kept under ICU Medical (project team confirmed ICU Medical / Smiths Medical is the manufacturer supplying India). Note for reference: graseby.com is now operated by Lianying Graseby Medical (China), and ICU's FY2025 10-K does not name Graseby.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Slide 2: reclassify Mindray 3 Series (SP3/VP3) to Smart - drug library present
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014jxHyvpwsKVbJ3RxrkkV1k
</commit_message>
<xml_diff>
--- a/Infusion_Pumps_India/Infusion_Pump_Classification_India_Slide2.xlsx
+++ b/Infusion_Pumps_India/Infusion_Pump_Classification_India_Slide2.xlsx
@@ -865,7 +865,7 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>BeneFusion 5 Series (SP5)**</t>
+          <t>BeneFusion 3 Series (SP3)</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>BeneFusion 5 Series (VP5)**</t>
+          <t>BeneFusion 3 Series (VP3)</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr">
@@ -892,8 +892,8 @@
         <is>
           <t>- 5 Series: Smart -&gt; Smart** (wireless module optional; DS5 dock)
 - e Series (eSP/eVP): Smart -&gt; Connected (DERS + wired/wireless CMS monitoring)
-- 1/3 Series Standard and u Series Connected confirmed
-- 3 Series has a 200-drug name list without dose limits: kept Standard (decision needed)</t>
+- 3 Series: Standard -&gt; Smart (data sheets show a small drug library, up to 200 drugs)
+- 1 Series Standard and u Series Connected confirmed</t>
         </is>
       </c>
     </row>
@@ -901,23 +901,23 @@
       <c r="A8" s="10" t="n"/>
       <c r="B8" s="10" t="n"/>
       <c r="C8" s="10" t="n"/>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>BeneFusion 3 Series (SP3)</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="n"/>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>BeneFusion 5 Series (SP5)**</t>
+        </is>
+      </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
           <t>BeneFusion u Series (uSP / uDSP)</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>BeneFusion 3 Series (VP3)</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="n"/>
+      <c r="G8" s="16" t="n"/>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>BeneFusion 5 Series (VP5)**</t>
+        </is>
+      </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
           <t>BeneFusion u Series (uVP)</t>
@@ -1530,37 +1530,37 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
+          <t>Smart</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>Official India website</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>https://www.mindray.com/in/products/infusion-system/benefusion-3-series/</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>SP3 data sheet (IndiaMart-hosted): https://5.imimg.com/data5/SELLER/Doc/2022/1/TX/CI/VD/17862303/mindray-benefusion-sp3-syringe-pump.pdf</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="G8" s="19" t="inlineStr">
-        <is>
-          <t>Official India website</t>
-        </is>
-      </c>
-      <c r="H8" s="20" t="inlineStr">
-        <is>
-          <t>https://www.mindray.com/in/products/infusion-system/benefusion-3-series/</t>
-        </is>
-      </c>
-      <c r="I8" s="13" t="inlineStr">
-        <is>
-          <t>SP3 data sheet (IndiaMart-hosted): https://5.imimg.com/data5/SELLER/Doc/2022/1/TX/CI/VD/17862303/mindray-benefusion-sp3-syringe-pump.pdf</t>
-        </is>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>Kept Standard - DECISION NEEDED (see note)</t>
+          <t>RECLASSIFY Standard -&gt; Smart (drug library present, per project team rule)</t>
         </is>
       </c>
       <c r="L8" s="13" t="inlineStr">
         <is>
-          <t>Judgement call: if a drug-NAME library without dose limits counts as a 'drug library', SP3/VP3 move to Smart. Kept Standard, as in the sample, because there are no dose limits (DERS).</t>
+          <t>Drug library is small (up to 200 drugs, ON/OFF switchable) and no dose limits (DERS) are stated, unlike the 5/e/u Series (up to 5,000 drugs with hard/soft limits). Classified Smart because a drug library is present (project team decision). No connectivity.</t>
         </is>
       </c>
       <c r="M8" s="13" t="inlineStr">
@@ -1597,37 +1597,37 @@
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
+          <t>Smart</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>Official India website</t>
+        </is>
+      </c>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>https://www.mindray.com/in/products/infusion-system/benefusion-3-series/</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>VP3 data sheet: https://alibenalimedical.com/wp-content/uploads/2025/11/BeneFusion-VP3_Datasheet_ENG_20210305%D9%85%D8%B6%D8%AE%D8%A9-%D9%85%D8%AD%D8%A7%D9%84%D9%8A%D9%84-.pdf | India page images show volumetric + syringe 3 Series pumps.</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="G9" s="19" t="inlineStr">
-        <is>
-          <t>Official India website</t>
-        </is>
-      </c>
-      <c r="H9" s="20" t="inlineStr">
-        <is>
-          <t>https://www.mindray.com/in/products/infusion-system/benefusion-3-series/</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr">
-        <is>
-          <t>India page hero/product images show volumetric + syringe 3 Series pumps.</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>Kept Standard - DECISION NEEDED (see note)</t>
+          <t>RECLASSIFY Standard -&gt; Smart (drug library present, per project team rule)</t>
         </is>
       </c>
       <c r="L9" s="13" t="inlineStr">
         <is>
-          <t>Same judgement call as SP3.</t>
+          <t>Same as SP3: small drug library (up to 200 drugs), no dose limits stated, no connectivity.</t>
         </is>
       </c>
       <c r="M9" s="13" t="inlineStr">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>Was missing from source list; Standard</t>
+          <t>Was missing from source list; Smart (drug library per data sheets)</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>'Drug library up to 200 drugs' - name list, no dose limits</t>
+          <t>'Drug library up to 200 drugs; ON/OFF switchable' (evidence for Smart)</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>4. Judgement call (Mindray 3 Series): data sheets show a drug-NAME library (up to 200 drugs) with no dose limits. Kept Standard, as in the sample; it moves to Smart if any drug library counts.</t>
+          <t>4. Mindray 3 Series: data sheets show a small drug library (up to 200 drugs, no dose limits stated). Classified Smart because a drug library is present (project team rule: any drug library = Smart).</t>
         </is>
       </c>
     </row>

</xml_diff>